<commit_message>
AKBO pricelist: update proposed descriptions to v3 brochure series names
Multi-Purpose -> Classic Plus, stainless Multi-Purpose -> Classic SS,
Lightweight -> Classic Lite, High-Flow -> Classic High-Flow, Hot-Water ->
Classic Hot Wash, ATEX -> Classic ATEX, Sterilisable -> Classic SS
Sterilisable (NozzleWorks_Brochures_2026-10-06_v3). AKRB001-BL flagged as
not covered by any brochure.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DBvGziJnByoD74uLTnaLZa
</commit_message>
<xml_diff>
--- a/pricelists/arbo/Nozzleworks_Pricelist_AKBO_washdown_guns.xlsx
+++ b/pricelists/arbo/Nozzleworks_Pricelist_AKBO_washdown_guns.xlsx
@@ -945,7 +945,7 @@
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>Lightweight water gun, w/o trigger guard, blue, PA66 plastic</t>
+          <t>Classic Lite water gun, w/o trigger guard, blue, PA66 plastic</t>
         </is>
       </c>
       <c r="E18" s="23" t="n">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="D29" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, blue, brass</t>
+          <t>Classic Plus water gun, w/o trigger guard, blue, brass</t>
         </is>
       </c>
       <c r="E29" s="23" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, red, brass</t>
+          <t>Classic Plus water gun, w/o trigger guard, red, brass</t>
         </is>
       </c>
       <c r="E30" s="23" t="n">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="D31" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, green, brass</t>
+          <t>Classic Plus water gun, w/o trigger guard, green, brass</t>
         </is>
       </c>
       <c r="E31" s="23" t="n">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, black, brass</t>
+          <t>Classic Plus water gun, w/o trigger guard, black, brass</t>
         </is>
       </c>
       <c r="E32" s="23" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="D33" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, yellow, brass</t>
+          <t>Classic Plus water gun, w/o trigger guard, yellow, brass</t>
         </is>
       </c>
       <c r="E33" s="23" t="n">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="D34" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, white, brass</t>
+          <t>Classic Plus water gun, w/o trigger guard, white, brass</t>
         </is>
       </c>
       <c r="E34" s="23" t="n">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="D35" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/ trigger guard, blue, brass</t>
+          <t>Classic Plus water gun, w/ trigger guard, blue, brass</t>
         </is>
       </c>
       <c r="E35" s="23" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="D36" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/ trigger guard, 1/2" F swivel, blue, brass</t>
+          <t>Classic Plus water gun, w/ trigger guard, 1/2" F swivel, blue, brass</t>
         </is>
       </c>
       <c r="E36" s="23" t="n">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="D37" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/ trigger guard, 3/4" F swivel, blue, brass</t>
+          <t>Classic Plus water gun, w/ trigger guard, 3/4" F swivel, blue, brass</t>
         </is>
       </c>
       <c r="E37" s="23" t="n">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="D44" s="22" t="inlineStr">
         <is>
-          <t>High-Flow water gun, w/o trigger guard, black, brass</t>
+          <t>Classic High-Flow water gun, w/o trigger guard, black, brass</t>
         </is>
       </c>
       <c r="E44" s="23" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D45" s="22" t="inlineStr">
         <is>
-          <t>High-Flow water gun, w/ trigger guard, black, brass</t>
+          <t>Classic High-Flow water gun, w/ trigger guard, black, brass</t>
         </is>
       </c>
       <c r="E45" s="30" t="n">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="D46" s="22" t="inlineStr">
         <is>
-          <t>High-Flow water gun, w/o trigger guard, black, stainless steel 316</t>
+          <t>Classic High-Flow water gun, w/o trigger guard, black, stainless steel 316</t>
         </is>
       </c>
       <c r="E46" s="30" t="n">
@@ -2588,7 +2588,7 @@
         <v/>
       </c>
       <c r="P46" s="29">
-        <f>TRIM(IF($B46="NOT ASSIGNED","No NW part no. ","")&amp;IFERROR(IF(INDEX(Conversion!$J$2:$J$500,MATCH($A46,Conversion!$B$2:$B$500,0))="Needs review","Conversion table: needs review. ",""),"")&amp;IF(LEFT($F46,8)="ESTIMATE","Weight estimated. ","")&amp;"")</f>
+        <f>TRIM(IF($B46="NOT ASSIGNED","No NW part no. ","")&amp;IFERROR(IF(INDEX(Conversion!$J$2:$J$500,MATCH($A46,Conversion!$B$2:$B$500,0))="Needs review","Conversion table: needs review. ",""),"")&amp;IF(LEFT($F46,8)="ESTIMATE","Weight estimated. ","")&amp;"Not in Classic High-Flow brochure (brass only) - series name to confirm.")</f>
         <v/>
       </c>
     </row>
@@ -2993,7 +2993,7 @@
       </c>
       <c r="D55" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, blue, stainless steel 316</t>
+          <t>Classic SS water gun, w/o trigger guard, blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E55" s="23" t="n">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="D56" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/o trigger guard, white, stainless steel 316</t>
+          <t>Classic SS water gun, w/o trigger guard, white, stainless steel 316</t>
         </is>
       </c>
       <c r="E56" s="23" t="n">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="D57" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/ trigger guard, blue, stainless steel 316</t>
+          <t>Classic SS water gun, w/ trigger guard, blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E57" s="23" t="n">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="D58" s="22" t="inlineStr">
         <is>
-          <t>Multi-Purpose water gun, w/ trigger guard, white, stainless steel 316</t>
+          <t>Classic SS water gun, w/ trigger guard, white, stainless steel 316</t>
         </is>
       </c>
       <c r="E58" s="23" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="D60" s="22" t="inlineStr">
         <is>
-          <t>Hot-Water gun, w/ trigger guard, Teflon/air insulated grip, red, stainless steel 316</t>
+          <t>Classic Hot Wash water gun, w/ trigger guard, Teflon/air insulated grip, red, stainless steel 316</t>
         </is>
       </c>
       <c r="E60" s="23" t="n">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="D61" s="22" t="inlineStr">
         <is>
-          <t>Hot-Water gun, w/ trigger guard, high flow, Teflon/air insulated grip, red, stainless steel 316</t>
+          <t>Classic Hot Wash water gun, w/ trigger guard, high flow, Teflon/air insulated grip, red, stainless steel 316</t>
         </is>
       </c>
       <c r="E61" s="23" t="n">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="D62" s="22" t="inlineStr">
         <is>
-          <t>Hot-Water gun, w/ trigger guard, 40 cm lance, Teflon/air insulated grip, red, stainless steel 316</t>
+          <t>Classic Hot Wash water gun, w/ trigger guard, 40 cm lance, Teflon/air insulated grip, red, stainless steel 316</t>
         </is>
       </c>
       <c r="E62" s="23" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="D64" s="22" t="inlineStr">
         <is>
-          <t>ATEX water gun, w/ trigger guard, Zone 1 &amp; 2, black, stainless steel 316</t>
+          <t>Classic ATEX water gun, w/ trigger guard, Zone 1 &amp; 2, black, stainless steel 316</t>
         </is>
       </c>
       <c r="E64" s="23" t="n">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="D65" s="22" t="inlineStr">
         <is>
-          <t>Sterilisable water gun, latex jacket, light blue, stainless steel 316</t>
+          <t>Classic SS Sterilisable water gun, latex jacket, light blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E65" s="23" t="n">
@@ -17041,7 +17041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C200"/>
+  <dimension ref="A1:C201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -19888,130 +19888,142 @@
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
         <is>
-          <t>AKMNP01-B-SW12</t>
+          <t>AKRB001-BL</t>
         </is>
       </c>
       <c r="C190" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Page 2 technical-data table header spells this "AKMP01-B-SW12" (missing N) - likely a table typo, confirm before use</t>
+          <t>Not in Classic High-Flow brochure (brass only) - series name to confirm.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
         <is>
-          <t>AKMNP01-B-SW34</t>
+          <t>AKMNP01-B-SW12</t>
         </is>
       </c>
       <c r="C191" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Page 2 technical-data table header spells this "AKMP01-B-SW34" (missing N) - likely a table typo, confirm before use</t>
+          <t>Conversion table: Page 2 technical-data table header spells this "AKMP01-B-SW12" (missing N) - likely a table typo, confirm before use</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
         <is>
-          <t>AKRB001-BL</t>
+          <t>AKMNP01-B-SW34</t>
         </is>
       </c>
       <c r="C192" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Page 12 cross-references this as the high-flow AISI316 variant ("full spec page 16"), but page 16 (High-flow cleaning guns) only lists brass "AKMB*" numbers - no matching AKRB* found there. Confirm actual model number with AKBO</t>
+          <t>Conversion table: Page 2 technical-data table header spells this "AKMP01-B-SW34" (missing N) - likely a table typo, confirm before use</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="inlineStr">
         <is>
-          <t>AKRHP01-R</t>
+          <t>AKRB001-BL</t>
         </is>
       </c>
       <c r="C193" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Body text calls the base model "AKRHP01-R" but the technical-data table heads its column "AKRHP02-R" - confirm which is correct with AKBO</t>
+          <t>Conversion table: Page 12 cross-references this as the high-flow AISI316 variant ("full spec page 16"), but page 16 (High-flow cleaning guns) only lists brass "AKMB*" numbers - no matching AKRB* found there. Confirm actual model number with AKBO</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="inlineStr">
         <is>
-          <t>AKRHP02-R-L40</t>
+          <t>AKRHP01-R</t>
         </is>
       </c>
       <c r="C194" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Table heading drops the "-R-" and reads "AKRHP02-L40" - confirm exact number with AKBO</t>
+          <t>Conversion table: Body text calls the base model "AKRHP01-R" but the technical-data table heads its column "AKRHP02-R" - confirm which is correct with AKBO</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="inlineStr">
         <is>
-          <t>BABTLF1-BL</t>
+          <t>AKRHP02-R-L40</t>
         </is>
       </c>
       <c r="C195" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Max-temp table cell shows "(231F)" matching a 95C row, but this model is rated 50C (its sibling BABTLF1-B-V, same 50C rating, correctly shows ~122F) - likely a copy-paste error in AKBO's table; confirm actual max temp with AKBO</t>
+          <t>Conversion table: Table heading drops the "-R-" and reads "AKRHP02-L40" - confirm exact number with AKBO</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
         <is>
-          <t>AKMSHHL1-BL</t>
+          <t>BABTLF1-BL</t>
         </is>
       </c>
       <c r="C196" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Technical-data table only lists dimensions/weight for the with-handle assemblies (AKMSHL1-B/AKRSHL1-B) - head-only weight not separately tabulated on this page</t>
+          <t>Conversion table: Max-temp table cell shows "(231F)" matching a 95C row, but this model is rated 50C (its sibling BABTLF1-B-V, same 50C rating, correctly shows ~122F) - likely a copy-paste error in AKBO's table; confirm actual max temp with AKBO</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
         <is>
-          <t>AKRSHHL1-BL</t>
+          <t>AKMSHHL1-BL</t>
         </is>
       </c>
       <c r="C197" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Technical-data table only lists dimensions/weight for the with-handle assemblies - head-only weight not separately tabulated on this page</t>
+          <t>Conversion table: Technical-data table only lists dimensions/weight for the with-handle assemblies (AKMSHL1-B/AKRSHL1-B) - head-only weight not separately tabulated on this page</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
         <is>
-          <t>AKRSHW3-W</t>
+          <t>AKRSHHL1-BL</t>
         </is>
       </c>
       <c r="C198" s="4" t="inlineStr">
         <is>
-          <t>Conversion table: Part number breaks the "03" pattern of its blue/red siblings (AKRSH03-B/R) - consistently printed as AKRSHW3-W in both body text and image caption, so likely intentional, but worth confirming with AKBO</t>
+          <t>Conversion table: Technical-data table only lists dimensions/weight for the with-handle assemblies - head-only weight not separately tabulated on this page</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
         <is>
-          <t>AGIL572 / AKAWLU1-B</t>
+          <t>AKRSHW3-W</t>
         </is>
       </c>
       <c r="C199" s="4" t="inlineStr">
         <is>
-          <t>AKBO show only one price plus a pack-qty note (48 pcs EUR 9.87 / 20 pcs EUR 66.81) - kept as note, not priced.</t>
+          <t>Conversion table: Part number breaks the "03" pattern of its blue/red siblings (AKRSH03-B/R) - consistently printed as AKRSHW3-W in both body text and image caption, so likely intentional, but worth confirming with AKBO</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
         <is>
+          <t>AGIL572 / AKAWLU1-B</t>
+        </is>
+      </c>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>AKBO show only one price plus a pack-qty note (48 pcs EUR 9.87 / 20 pcs EUR 66.81) - kept as note, not priced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
           <t>Heavy duty spray guns</t>
         </is>
       </c>
-      <c r="C200" s="4" t="inlineStr">
+      <c r="C201" s="4" t="inlineStr">
         <is>
           <t>AKBO give no &gt;=50 pcs price for most guns - left blank.</t>
         </is>

</xml_diff>

<commit_message>
AKBO pricelist: use 'WD gun' instead of 'water gun' in proposed descriptions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DBvGziJnByoD74uLTnaLZa
</commit_message>
<xml_diff>
--- a/pricelists/arbo/Nozzleworks_Pricelist_AKBO_washdown_guns.xlsx
+++ b/pricelists/arbo/Nozzleworks_Pricelist_AKBO_washdown_guns.xlsx
@@ -945,7 +945,7 @@
       </c>
       <c r="D18" s="22" t="inlineStr">
         <is>
-          <t>Classic Lite water gun, w/o trigger guard, blue, PA66 plastic</t>
+          <t>Classic Lite WD gun, w/o trigger guard, blue, PA66 plastic</t>
         </is>
       </c>
       <c r="E18" s="23" t="n">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="D19" s="22" t="inlineStr">
         <is>
-          <t>Blue Princess water gun, w/o trigger guard, blue, brass</t>
+          <t>Blue Princess WD gun, w/o trigger guard, blue, brass</t>
         </is>
       </c>
       <c r="E19" s="23" t="n">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>Blue Princess water gun, w/o trigger guard, PRINCESS logo, blue, brass</t>
+          <t>Blue Princess WD gun, w/o trigger guard, PRINCESS logo, blue, brass</t>
         </is>
       </c>
       <c r="E20" s="23" t="n">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="D21" s="22" t="inlineStr">
         <is>
-          <t>Blue Princess water gun, w/ trigger guard, PRINCESS logo, blue, brass</t>
+          <t>Blue Princess WD gun, w/ trigger guard, PRINCESS logo, blue, brass</t>
         </is>
       </c>
       <c r="E21" s="23" t="n">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="D22" s="22" t="inlineStr">
         <is>
-          <t>Classic water gun, w/o trigger insulation, blue, brass</t>
+          <t>Classic WD gun, w/o trigger insulation, blue, brass</t>
         </is>
       </c>
       <c r="E22" s="23" t="n">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="D23" s="22" t="inlineStr">
         <is>
-          <t>Classic water gun, w/o trigger insulation, red, brass</t>
+          <t>Classic WD gun, w/o trigger insulation, red, brass</t>
         </is>
       </c>
       <c r="E23" s="23" t="n">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>Classic water gun, w/o trigger insulation, green, brass</t>
+          <t>Classic WD gun, w/o trigger insulation, green, brass</t>
         </is>
       </c>
       <c r="E24" s="23" t="n">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="D25" s="22" t="inlineStr">
         <is>
-          <t>Classic water gun, w/o trigger insulation, black, brass</t>
+          <t>Classic WD gun, w/o trigger insulation, black, brass</t>
         </is>
       </c>
       <c r="E25" s="23" t="n">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
-          <t>Classic water gun, w/o trigger insulation, yellow, brass</t>
+          <t>Classic WD gun, w/o trigger insulation, yellow, brass</t>
         </is>
       </c>
       <c r="E26" s="23" t="n">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="D27" s="22" t="inlineStr">
         <is>
-          <t>Classic water gun, w/o trigger insulation, white, brass</t>
+          <t>Classic WD gun, w/o trigger insulation, white, brass</t>
         </is>
       </c>
       <c r="E27" s="23" t="n">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="D29" s="22" t="inlineStr">
         <is>
-          <t>Classic Plus water gun, w/o trigger guard, blue, brass</t>
+          <t>Classic Plus WD gun, w/o trigger guard, blue, brass</t>
         </is>
       </c>
       <c r="E29" s="23" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="D30" s="22" t="inlineStr">
         <is>
-          <t>Classic Plus water gun, w/o trigger guard, red, brass</t>
+          <t>Classic Plus WD gun, w/o trigger guard, red, brass</t>
         </is>
       </c>
       <c r="E30" s="23" t="n">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="D31" s="22" t="inlineStr">
         <is>
-          <t>Classic Plus water gun, w/o trigger guard, green, brass</t>
+          <t>Classic Plus WD gun, w/o trigger guard, green, brass</t>
         </is>
       </c>
       <c r="E31" s="23" t="n">
@@ -1777,7 +1777,7 @@
       </c>
       <c r="D32" s="22" t="inlineStr">
         <is>
-          <t>Classic Plus water gun, w/o trigger guard, black, brass</t>
+          <t>Classic Plus WD gun, w/o trigger guard, black, brass</t>
         </is>
       </c>
       <c r="E32" s="23" t="n">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="D33" s="22" t="inlineStr">
         <is>
-          <t>Classic Plus water gun, w/o trigger guard, yellow, brass</t>
+          <t>Classic Plus WD gun, w/o trigger guard, yellow, brass</t>
         </is>
       </c>
       <c r="E33" s="23" t="n">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="D34" s="22" t="inlineStr">
         <is>
-          <t>Classic Plus water gun, w/o trigger guard, white, brass</t>
+          <t>Classic Plus WD gun, w/o trigger guard, white, brass</t>
         </is>
       </c>
       <c r="E34" s="23" t="n">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="D35" s="22" t="inlineStr">
         <is>
-          <t>Classic Plus water gun, w/ trigger guard, blue, brass</t>
+          <t>Classic Plus WD gun, w/ trigger guard, blue, brass</t>
         </is>
       </c>
       <c r="E35" s="23" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="D37" s="22" t="inlineStr">
         <is>
-          <t>Blue King water gun, w/o trigger guard, blue, brass</t>
+          <t>Blue King WD gun, w/o trigger guard, blue, brass</t>
         </is>
       </c>
       <c r="E37" s="23" t="n">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="D38" s="22" t="inlineStr">
         <is>
-          <t>Blue King water gun, w/o trigger guard, KING logo, blue, brass</t>
+          <t>Blue King WD gun, w/o trigger guard, KING logo, blue, brass</t>
         </is>
       </c>
       <c r="E38" s="23" t="n">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="D39" s="22" t="inlineStr">
         <is>
-          <t>Blue King water gun, w/ trigger guard, blue, brass</t>
+          <t>Blue King WD gun, w/ trigger guard, blue, brass</t>
         </is>
       </c>
       <c r="E39" s="23" t="n">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D40" s="22" t="inlineStr">
         <is>
-          <t>Blue King water gun, w/ trigger guard, KING logo, blue, brass</t>
+          <t>Blue King WD gun, w/ trigger guard, KING logo, blue, brass</t>
         </is>
       </c>
       <c r="E40" s="23" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="D42" s="22" t="inlineStr">
         <is>
-          <t>Classic High-Flow water gun, w/o trigger guard, black, brass</t>
+          <t>Classic High-Flow WD gun, w/o trigger guard, black, brass</t>
         </is>
       </c>
       <c r="E42" s="23" t="n">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="D43" s="22" t="inlineStr">
         <is>
-          <t>Classic High-Flow water gun, w/ trigger guard, black, brass</t>
+          <t>Classic High-Flow WD gun, w/ trigger guard, black, brass</t>
         </is>
       </c>
       <c r="E43" s="30" t="n">
@@ -2417,7 +2417,7 @@
       </c>
       <c r="D44" s="22" t="inlineStr">
         <is>
-          <t>Classic High-Flow water gun, w/o trigger guard, black, stainless steel 316</t>
+          <t>Classic High-Flow WD gun, w/o trigger guard, black, stainless steel 316</t>
         </is>
       </c>
       <c r="E44" s="30" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D46" s="22" t="inlineStr">
         <is>
-          <t>Classic Protection Plus water gun, w/o trigger guard, blue, chrome-plated brass</t>
+          <t>Classic Protection Plus WD gun, w/o trigger guard, blue, chrome-plated brass</t>
         </is>
       </c>
       <c r="E46" s="23" t="n">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="D47" s="22" t="inlineStr">
         <is>
-          <t>Classic Protection Plus water gun, w/ trigger guard, blue, chrome-plated brass</t>
+          <t>Classic Protection Plus WD gun, w/ trigger guard, blue, chrome-plated brass</t>
         </is>
       </c>
       <c r="E47" s="23" t="n">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="D48" s="22" t="inlineStr">
         <is>
-          <t>Classic Protection Plus water gun, w/ trigger guard, white, chrome-plated brass</t>
+          <t>Classic Protection Plus WD gun, w/ trigger guard, white, chrome-plated brass</t>
         </is>
       </c>
       <c r="E48" s="23" t="n">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="D50" s="22" t="inlineStr">
         <is>
-          <t>Blue Princess water gun, w/o trigger guard, blue, stainless steel 316</t>
+          <t>Blue Princess WD gun, w/o trigger guard, blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E50" s="23" t="n">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="D51" s="22" t="inlineStr">
         <is>
-          <t>Blue Princess water gun, w/o trigger guard, PRINCESS logo, blue, stainless steel 316</t>
+          <t>Blue Princess WD gun, w/o trigger guard, PRINCESS logo, blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E51" s="23" t="n">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="D52" s="22" t="inlineStr">
         <is>
-          <t>Blue Princess water gun, w/ trigger guard, PRINCESS logo, blue, stainless steel 316</t>
+          <t>Blue Princess WD gun, w/ trigger guard, PRINCESS logo, blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E52" s="23" t="n">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="D53" s="22" t="inlineStr">
         <is>
-          <t>Classic SS water gun, w/o trigger guard, blue, stainless steel 316</t>
+          <t>Classic SS WD gun, w/o trigger guard, blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E53" s="23" t="n">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="D54" s="22" t="inlineStr">
         <is>
-          <t>Classic SS water gun, w/o trigger guard, white, stainless steel 316</t>
+          <t>Classic SS WD gun, w/o trigger guard, white, stainless steel 316</t>
         </is>
       </c>
       <c r="E54" s="23" t="n">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="D55" s="22" t="inlineStr">
         <is>
-          <t>Classic SS water gun, w/ trigger guard, blue, stainless steel 316</t>
+          <t>Classic SS WD gun, w/ trigger guard, blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E55" s="23" t="n">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="D56" s="22" t="inlineStr">
         <is>
-          <t>Classic SS water gun, w/ trigger guard, white, stainless steel 316</t>
+          <t>Classic SS WD gun, w/ trigger guard, white, stainless steel 316</t>
         </is>
       </c>
       <c r="E56" s="23" t="n">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="D58" s="22" t="inlineStr">
         <is>
-          <t>Classic Hot Wash water gun, w/ trigger guard, Teflon/air insulated grip, red, stainless steel 316</t>
+          <t>Classic Hot Wash WD gun, w/ trigger guard, Teflon/air insulated grip, red, stainless steel 316</t>
         </is>
       </c>
       <c r="E58" s="23" t="n">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="D59" s="22" t="inlineStr">
         <is>
-          <t>Classic Hot Wash water gun, w/ trigger guard, high flow, Teflon/air insulated grip, red, stainless steel 316</t>
+          <t>Classic Hot Wash WD gun, w/ trigger guard, high flow, Teflon/air insulated grip, red, stainless steel 316</t>
         </is>
       </c>
       <c r="E59" s="23" t="n">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="D60" s="22" t="inlineStr">
         <is>
-          <t>Classic Hot Wash water gun, w/ trigger guard, 40 cm lance, Teflon/air insulated grip, red, stainless steel 316</t>
+          <t>Classic Hot Wash WD gun, w/ trigger guard, 40 cm lance, Teflon/air insulated grip, red, stainless steel 316</t>
         </is>
       </c>
       <c r="E60" s="23" t="n">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="D62" s="22" t="inlineStr">
         <is>
-          <t>Classic ATEX water gun, w/ trigger guard, Zone 1 &amp; 2, black, stainless steel 316</t>
+          <t>Classic ATEX WD gun, w/ trigger guard, Zone 1 &amp; 2, black, stainless steel 316</t>
         </is>
       </c>
       <c r="E62" s="23" t="n">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="D63" s="22" t="inlineStr">
         <is>
-          <t>Classic SS Sterilisable water gun, latex jacket, light blue, stainless steel 316</t>
+          <t>Classic SS Sterilisable WD gun, latex jacket, light blue, stainless steel 316</t>
         </is>
       </c>
       <c r="E63" s="23" t="n">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="D73" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, blue, aluminium</t>
+          <t>Baby WD gun, rear trigger, blue, aluminium</t>
         </is>
       </c>
       <c r="E73" s="23" t="n">
@@ -3727,7 +3727,7 @@
       </c>
       <c r="D74" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, 1/2" F outlet, black, aluminium</t>
+          <t>Baby WD gun, rear trigger, 1/2" F outlet, black, aluminium</t>
         </is>
       </c>
       <c r="E74" s="23" t="n">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="D75" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, adapter outlet, blue, aluminium</t>
+          <t>Baby WD gun, rear trigger, adapter outlet, blue, aluminium</t>
         </is>
       </c>
       <c r="E75" s="30" t="n">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="D76" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, adapter inlet &amp; outlet, blue, aluminium</t>
+          <t>Baby WD gun, rear trigger, adapter inlet &amp; outlet, blue, aluminium</t>
         </is>
       </c>
       <c r="E76" s="30" t="n">
@@ -3941,7 +3941,7 @@
       </c>
       <c r="D80" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, blue, brass</t>
+          <t>Baby WD gun, rear trigger, blue, brass</t>
         </is>
       </c>
       <c r="E80" s="23" t="n">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="D81" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, 1/2" M outlet, adjustable nozzle, blue, brass</t>
+          <t>Baby WD gun, rear trigger, 1/2" M outlet, adjustable nozzle, blue, brass</t>
         </is>
       </c>
       <c r="E81" s="23" t="n">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="D82" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, 1/2" M outlet, blue, brass</t>
+          <t>Baby WD gun, rear trigger, 1/2" M outlet, blue, brass</t>
         </is>
       </c>
       <c r="E82" s="30" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="D83" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, adapter outlet, blue, brass</t>
+          <t>Baby WD gun, rear trigger, adapter outlet, blue, brass</t>
         </is>
       </c>
       <c r="E83" s="30" t="n">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="D84" s="22" t="inlineStr">
         <is>
-          <t>Baby water gun, rear trigger, adapter outlet, Viton seals, blue, brass</t>
+          <t>Baby WD gun, rear trigger, adapter outlet, Viton seals, blue, brass</t>
         </is>
       </c>
       <c r="E84" s="30" t="n">
@@ -5657,7 +5657,7 @@
       </c>
       <c r="D115" s="22" t="inlineStr">
         <is>
-          <t>Air-Boosted water gun, 2x 10 mm hose tails (air &amp; water), blue, aluminium</t>
+          <t>Air-Boosted WD gun, 2x 10 mm hose tails (air &amp; water), blue, aluminium</t>
         </is>
       </c>
       <c r="E115" s="23" t="n">

</xml_diff>